<commit_message>
Fix collections % to use prior-month billings; wire Amplia collections
- Collections_Pct now reads Prior_Month_Collections_Pct from the sheet
  (collections vs prior month's billings) instead of incorrectly dividing
  by the current month's billings
- Amplia collections and percentage are now read from Collections_Billing
  instead of being hardcoded to None ("Data pending")

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Master_Data_Template.xlsx
+++ b/TSTT_Master_Data_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tsttcott-my.sharepoint.com/personal/csimeon_tstt_co_tt/Documents/Financial Analysis/TSTT_Board_Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="11_6F8991EE5281D36470E2DCD46D0A78F2D2E811F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4FCE522-6223-4598-A5B0-609A5665073B}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="11_6F8991EE5281D36470E2DCD46D0A78F2D2E811F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB22F2A4-651A-47CF-BE85-C1059B8B5F2A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="Prepaid_Data_Usage" sheetId="14" r:id="rId14"/>
     <sheet name="Postpaid by active Plan" sheetId="15" r:id="rId15"/>
     <sheet name="WTTX by Category" sheetId="16" r:id="rId16"/>
+    <sheet name="Business_Sales_MRR" sheetId="17" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'P&amp;L_Segments'!$A$3:$P$128</definedName>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3460" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3691" uniqueCount="504">
   <si>
     <t>TSTT BOARD REPORT — MASTER DATA FILE</t>
   </si>
@@ -1485,6 +1486,87 @@
   </si>
   <si>
     <t>MOBILE</t>
+  </si>
+  <si>
+    <t>Apr 2025</t>
+  </si>
+  <si>
+    <t>May 2025</t>
+  </si>
+  <si>
+    <t>Jun 2025</t>
+  </si>
+  <si>
+    <t>Jul 2025</t>
+  </si>
+  <si>
+    <t>Aug 2025</t>
+  </si>
+  <si>
+    <t>Sep 2025</t>
+  </si>
+  <si>
+    <t>Oct 2025</t>
+  </si>
+  <si>
+    <t>Nov 2025</t>
+  </si>
+  <si>
+    <t>Dec 2025</t>
+  </si>
+  <si>
+    <t>Jan 2026</t>
+  </si>
+  <si>
+    <t>Feb 2026</t>
+  </si>
+  <si>
+    <t>Mar 2026</t>
+  </si>
+  <si>
+    <t>Apr 2026</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>May-26</t>
+  </si>
+  <si>
+    <t>Jun-26</t>
+  </si>
+  <si>
+    <t>Jul-26</t>
+  </si>
+  <si>
+    <t>Aug-26</t>
+  </si>
+  <si>
+    <t>Sep-26</t>
+  </si>
+  <si>
+    <t>Oct-26</t>
+  </si>
+  <si>
+    <t>Nov-26</t>
+  </si>
+  <si>
+    <t>Dec-26</t>
+  </si>
+  <si>
+    <t>Jan-27</t>
+  </si>
+  <si>
+    <t>Feb-27</t>
+  </si>
+  <si>
+    <t>Mar-27</t>
   </si>
 </sst>
 </file>
@@ -1495,7 +1577,7 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1605,6 +1687,17 @@
     <font>
       <sz val="11"/>
       <name val="Candara"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1734,11 +1827,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1810,11 +1905,15 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1832,10 +1931,10 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1848,9 +1947,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{F2EBC6C1-47DC-40B1-8FA2-02F247C39251}"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2161,10 +2262,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="40"/>
+      <c r="A1" s="48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="44"/>
     </row>
     <row r="2" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2173,10 +2274,10 @@
       <c r="B2" s="2"/>
     </row>
     <row r="4" spans="1:2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="40"/>
+      <c r="B4" s="44"/>
     </row>
     <row r="5" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -2227,10 +2328,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="40"/>
+      <c r="B12" s="44"/>
     </row>
     <row r="13" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -2337,10 +2438,10 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="40"/>
+      <c r="B27" s="44"/>
     </row>
     <row r="28" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
@@ -2440,20 +2541,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="53" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:4" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="3" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -5996,28 +6097,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="53" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>204</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -6101,32 +6202,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="54" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>218</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
@@ -6215,22 +6316,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="55" t="s">
         <v>237</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>238</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
@@ -7050,26 +7151,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="55" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>249</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
@@ -9754,6 +9855,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F06867E-D865-4B23-9C8A-6E4BEE115DA3}">
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="39"/>
+    <col min="2" max="14" width="10.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="39"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B1" s="39" t="s">
+        <v>477</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>478</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>479</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>480</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G1" s="39" t="s">
+        <v>482</v>
+      </c>
+      <c r="H1" s="39" t="s">
+        <v>483</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>484</v>
+      </c>
+      <c r="J1" s="39" t="s">
+        <v>485</v>
+      </c>
+      <c r="K1" s="39" t="s">
+        <v>486</v>
+      </c>
+      <c r="L1" s="39" t="s">
+        <v>487</v>
+      </c>
+      <c r="M1" s="39" t="s">
+        <v>488</v>
+      </c>
+      <c r="N1" s="39" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="39" t="s">
+        <v>490</v>
+      </c>
+      <c r="B2" s="40">
+        <v>10103630</v>
+      </c>
+      <c r="C2" s="40">
+        <v>10284929</v>
+      </c>
+      <c r="D2" s="40">
+        <v>10196405</v>
+      </c>
+      <c r="E2" s="40">
+        <v>10399167</v>
+      </c>
+      <c r="F2" s="40">
+        <v>10123637</v>
+      </c>
+      <c r="G2" s="40">
+        <v>10330353</v>
+      </c>
+      <c r="H2" s="40">
+        <v>10280450</v>
+      </c>
+      <c r="I2" s="40">
+        <v>10433823</v>
+      </c>
+      <c r="J2" s="40">
+        <v>10370640</v>
+      </c>
+      <c r="K2" s="40">
+        <v>9957871</v>
+      </c>
+      <c r="L2" s="40">
+        <v>10773562</v>
+      </c>
+      <c r="M2" s="40">
+        <v>10261754</v>
+      </c>
+      <c r="N2" s="40">
+        <v>10388046</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="39" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="40">
+        <v>29246684.200000003</v>
+      </c>
+      <c r="C3" s="40">
+        <v>30137908.66</v>
+      </c>
+      <c r="D3" s="40">
+        <v>29672656.27</v>
+      </c>
+      <c r="E3" s="40">
+        <v>30013611.75</v>
+      </c>
+      <c r="F3" s="40">
+        <v>29783064.919999994</v>
+      </c>
+      <c r="G3" s="40">
+        <v>28978837.339999989</v>
+      </c>
+      <c r="H3" s="40">
+        <v>28498077.119999994</v>
+      </c>
+      <c r="I3" s="40">
+        <v>29393899.420000002</v>
+      </c>
+      <c r="J3" s="40">
+        <v>29497354.730000004</v>
+      </c>
+      <c r="K3" s="40">
+        <v>29235353.390000001</v>
+      </c>
+      <c r="L3" s="40">
+        <v>28522268.300000001</v>
+      </c>
+      <c r="M3" s="40">
+        <v>30332651.329999991</v>
+      </c>
+      <c r="N3" s="40">
+        <v>28727718.040000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
+        <v>491</v>
+      </c>
+      <c r="B4" s="40">
+        <v>6228573.3000000007</v>
+      </c>
+      <c r="C4" s="40">
+        <v>5307783.1099999994</v>
+      </c>
+      <c r="D4" s="40">
+        <v>5272540.34</v>
+      </c>
+      <c r="E4" s="40">
+        <v>5082307.5600000005</v>
+      </c>
+      <c r="F4" s="40">
+        <v>5109971.28</v>
+      </c>
+      <c r="G4" s="40">
+        <v>5127801.24</v>
+      </c>
+      <c r="H4" s="40">
+        <v>5768038.7200000007</v>
+      </c>
+      <c r="I4" s="40">
+        <v>5770776.1099999994</v>
+      </c>
+      <c r="J4" s="40">
+        <v>5423163.1400000006</v>
+      </c>
+      <c r="K4" s="40">
+        <v>5265592.2799999993</v>
+      </c>
+      <c r="L4" s="40">
+        <v>4232223.7699999996</v>
+      </c>
+      <c r="M4" s="40">
+        <v>4703865.1599999992</v>
+      </c>
+      <c r="N4" s="40">
+        <v>4143701.91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="39" t="s">
+        <v>475</v>
+      </c>
+      <c r="B5" s="40">
+        <v>1905399.38</v>
+      </c>
+      <c r="C5" s="40">
+        <v>2142482.52</v>
+      </c>
+      <c r="D5" s="40">
+        <v>3604616.9499999997</v>
+      </c>
+      <c r="E5" s="40">
+        <v>398517.42</v>
+      </c>
+      <c r="F5" s="40">
+        <v>3742714.2</v>
+      </c>
+      <c r="G5" s="40">
+        <v>3975131.08</v>
+      </c>
+      <c r="H5" s="40">
+        <v>3426313.79</v>
+      </c>
+      <c r="I5" s="40">
+        <v>2180647.08</v>
+      </c>
+      <c r="J5" s="40">
+        <v>8726744.2200000007</v>
+      </c>
+      <c r="K5" s="40">
+        <v>1998643.21</v>
+      </c>
+      <c r="L5" s="40">
+        <v>5153187.4699999988</v>
+      </c>
+      <c r="M5" s="40">
+        <v>1139632.75</v>
+      </c>
+      <c r="N5" s="40">
+        <v>8488566.7200000007</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
+        <v>492</v>
+      </c>
+      <c r="B6" s="40">
+        <v>47484286.880000003</v>
+      </c>
+      <c r="C6" s="40">
+        <v>47873103.289999999</v>
+      </c>
+      <c r="D6" s="40">
+        <v>48746218.560000002</v>
+      </c>
+      <c r="E6" s="40">
+        <v>45893603.730000004</v>
+      </c>
+      <c r="F6" s="40">
+        <v>48759387.399999999</v>
+      </c>
+      <c r="G6" s="40">
+        <v>48412122.659999989</v>
+      </c>
+      <c r="H6" s="40">
+        <v>47972879.629999988</v>
+      </c>
+      <c r="I6" s="40">
+        <v>47779145.609999999</v>
+      </c>
+      <c r="J6" s="40">
+        <v>54017902.090000004</v>
+      </c>
+      <c r="K6" s="40">
+        <v>46457459.880000003</v>
+      </c>
+      <c r="L6" s="40">
+        <v>48681241.539999992</v>
+      </c>
+      <c r="M6" s="40">
+        <v>46437903.239999987</v>
+      </c>
+      <c r="N6" s="40">
+        <v>51748032.670000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
@@ -9769,44 +10146,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
     </row>
     <row r="2" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
     </row>
     <row r="3" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -10967,6 +11344,9 @@
       <c r="F68">
         <v>-1834298</v>
       </c>
+      <c r="L68">
+        <v>70625668.580000043</v>
+      </c>
       <c r="N68">
         <v>14592872.859999999</v>
       </c>
@@ -11955,8 +12335,17 @@
       <c r="E124">
         <v>86147360.219999999</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="13">
         <v>14797376.029999999</v>
+      </c>
+      <c r="G124" s="13">
+        <v>9399347.083717268</v>
+      </c>
+      <c r="H124">
+        <v>88803389.900000006</v>
+      </c>
+      <c r="I124">
+        <v>80274532.463603497</v>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.25">
@@ -11975,8 +12364,17 @@
       <c r="E125">
         <v>50200295.450000003</v>
       </c>
-      <c r="F125">
+      <c r="F125" s="13">
         <v>7551484.3600000003</v>
+      </c>
+      <c r="G125" s="13">
+        <v>4924417.2113424698</v>
+      </c>
+      <c r="H125">
+        <v>51748032.659999989</v>
+      </c>
+      <c r="I125">
+        <v>46530148.564534202</v>
       </c>
     </row>
     <row r="126" spans="1:15" x14ac:dyDescent="0.25">
@@ -11995,8 +12393,17 @@
       <c r="E126">
         <v>905341.23</v>
       </c>
-      <c r="F126">
+      <c r="F126" s="13">
         <v>194375</v>
+      </c>
+      <c r="G126" s="13">
+        <v>215775.25</v>
+      </c>
+      <c r="H126">
+        <v>933254.02000000014</v>
+      </c>
+      <c r="I126">
+        <v>936088.9</v>
       </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.25">
@@ -12015,8 +12422,17 @@
       <c r="E127">
         <v>27726936.300000001</v>
       </c>
-      <c r="F127">
+      <c r="F127" s="13">
         <v>4556077.53</v>
+      </c>
+      <c r="G127" s="13">
+        <v>5142998.3076690342</v>
+      </c>
+      <c r="H127">
+        <v>28581792.039999995</v>
+      </c>
+      <c r="I127">
+        <v>28894159.209127802</v>
       </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.25">
@@ -12035,8 +12451,29 @@
       <c r="E128">
         <v>-3466351.67</v>
       </c>
-      <c r="F128">
+      <c r="F128" s="13">
         <v>-73002.539999999994</v>
+      </c>
+      <c r="G128" s="13">
+        <v>-2217682.8665</v>
+      </c>
+      <c r="H128">
+        <v>-3573223.5800000131</v>
+      </c>
+      <c r="I128">
+        <v>-2953301.1165000005</v>
+      </c>
+      <c r="J128">
+        <v>59863342.810000002</v>
+      </c>
+      <c r="K128">
+        <v>79146702.948436171</v>
+      </c>
+      <c r="L128">
+        <v>80592075.969999999</v>
+      </c>
+      <c r="M128">
+        <v>57125083.916100591</v>
       </c>
       <c r="N128">
         <v>21926019.510000002</v>
@@ -12060,7 +12497,7 @@
   <sheetPr>
     <tabColor rgb="FF196127"/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F218"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -12070,24 +12507,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="50" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -14129,7 +14566,7 @@
         <v>19029674.210000001</v>
       </c>
       <c r="E147">
-        <v>21277967.280000001</v>
+        <v>21277967.281142484</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
@@ -14194,10 +14631,10 @@
         <v>95</v>
       </c>
       <c r="D151">
-        <v>9390447.5399999991</v>
+        <v>13488346.060000002</v>
       </c>
       <c r="E151">
-        <v>17449675.469999999</v>
+        <v>24087604.517293684</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
@@ -14215,6 +14652,930 @@
       </c>
       <c r="E152">
         <v>3641316.3</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>493</v>
+      </c>
+      <c r="B153" t="s">
+        <v>90</v>
+      </c>
+      <c r="C153" t="s">
+        <v>98</v>
+      </c>
+      <c r="E153">
+        <v>22591612.332703259</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>493</v>
+      </c>
+      <c r="B154" t="s">
+        <v>90</v>
+      </c>
+      <c r="C154" t="s">
+        <v>91</v>
+      </c>
+      <c r="E154">
+        <v>23147297.862746108</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>493</v>
+      </c>
+      <c r="B155" t="s">
+        <v>90</v>
+      </c>
+      <c r="C155" t="s">
+        <v>94</v>
+      </c>
+      <c r="E155">
+        <v>14332013.6352381</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>493</v>
+      </c>
+      <c r="B156" t="s">
+        <v>90</v>
+      </c>
+      <c r="C156" t="s">
+        <v>95</v>
+      </c>
+      <c r="E156">
+        <v>17646306.05536446</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>493</v>
+      </c>
+      <c r="B157" t="s">
+        <v>90</v>
+      </c>
+      <c r="C157" t="s">
+        <v>96</v>
+      </c>
+      <c r="E157">
+        <v>3168047.0304404469</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>493</v>
+      </c>
+      <c r="B158" t="s">
+        <v>90</v>
+      </c>
+      <c r="C158" t="s">
+        <v>93</v>
+      </c>
+      <c r="E158">
+        <v>3241953.2328955359</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>494</v>
+      </c>
+      <c r="B159" t="s">
+        <v>90</v>
+      </c>
+      <c r="C159" t="s">
+        <v>98</v>
+      </c>
+      <c r="E159">
+        <v>22522911.54131892</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>494</v>
+      </c>
+      <c r="B160" t="s">
+        <v>90</v>
+      </c>
+      <c r="C160" t="s">
+        <v>91</v>
+      </c>
+      <c r="E160">
+        <v>23871463.000562731</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>494</v>
+      </c>
+      <c r="B161" t="s">
+        <v>90</v>
+      </c>
+      <c r="C161" t="s">
+        <v>94</v>
+      </c>
+      <c r="E161">
+        <v>17173048.7052381</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>494</v>
+      </c>
+      <c r="B162" t="s">
+        <v>90</v>
+      </c>
+      <c r="C162" t="s">
+        <v>95</v>
+      </c>
+      <c r="E162">
+        <v>19474521.734445091</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>494</v>
+      </c>
+      <c r="B163" t="s">
+        <v>90</v>
+      </c>
+      <c r="C163" t="s">
+        <v>96</v>
+      </c>
+      <c r="E163">
+        <v>3294321.1456401451</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>494</v>
+      </c>
+      <c r="B164" t="s">
+        <v>90</v>
+      </c>
+      <c r="C164" t="s">
+        <v>93</v>
+      </c>
+      <c r="E164">
+        <v>5201350.3279076247</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>495</v>
+      </c>
+      <c r="B165" t="s">
+        <v>90</v>
+      </c>
+      <c r="C165" t="s">
+        <v>98</v>
+      </c>
+      <c r="E165">
+        <v>22657637.09599318</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>495</v>
+      </c>
+      <c r="B166" t="s">
+        <v>90</v>
+      </c>
+      <c r="C166" t="s">
+        <v>91</v>
+      </c>
+      <c r="E166">
+        <v>22771503.687049419</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>495</v>
+      </c>
+      <c r="B167" t="s">
+        <v>90</v>
+      </c>
+      <c r="C167" t="s">
+        <v>94</v>
+      </c>
+      <c r="E167">
+        <v>15169612.6352381</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>495</v>
+      </c>
+      <c r="B168" t="s">
+        <v>90</v>
+      </c>
+      <c r="C168" t="s">
+        <v>95</v>
+      </c>
+      <c r="E168">
+        <v>110707370.97098359</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>495</v>
+      </c>
+      <c r="B169" t="s">
+        <v>90</v>
+      </c>
+      <c r="C169" t="s">
+        <v>96</v>
+      </c>
+      <c r="E169">
+        <v>3725840.471526688</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>495</v>
+      </c>
+      <c r="B170" t="s">
+        <v>90</v>
+      </c>
+      <c r="C170" t="s">
+        <v>93</v>
+      </c>
+      <c r="E170">
+        <v>2842128.7220176449</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>496</v>
+      </c>
+      <c r="B171" t="s">
+        <v>90</v>
+      </c>
+      <c r="C171" t="s">
+        <v>98</v>
+      </c>
+      <c r="E171">
+        <v>22986653.214691199</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>496</v>
+      </c>
+      <c r="B172" t="s">
+        <v>90</v>
+      </c>
+      <c r="C172" t="s">
+        <v>91</v>
+      </c>
+      <c r="E172">
+        <v>23101642.49688293</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>496</v>
+      </c>
+      <c r="B173" t="s">
+        <v>90</v>
+      </c>
+      <c r="C173" t="s">
+        <v>94</v>
+      </c>
+      <c r="E173">
+        <v>14093039.44476191</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>496</v>
+      </c>
+      <c r="B174" t="s">
+        <v>90</v>
+      </c>
+      <c r="C174" t="s">
+        <v>95</v>
+      </c>
+      <c r="E174">
+        <v>18031437.184675042</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>496</v>
+      </c>
+      <c r="B175" t="s">
+        <v>90</v>
+      </c>
+      <c r="C175" t="s">
+        <v>96</v>
+      </c>
+      <c r="E175">
+        <v>3794023.364505047</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>496</v>
+      </c>
+      <c r="B176" t="s">
+        <v>90</v>
+      </c>
+      <c r="C176" t="s">
+        <v>93</v>
+      </c>
+      <c r="E176">
+        <v>4722333.8230922902</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>497</v>
+      </c>
+      <c r="B177" t="s">
+        <v>90</v>
+      </c>
+      <c r="C177" t="s">
+        <v>98</v>
+      </c>
+      <c r="E177">
+        <v>22449175.764702048</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>497</v>
+      </c>
+      <c r="B178" t="s">
+        <v>90</v>
+      </c>
+      <c r="C178" t="s">
+        <v>91</v>
+      </c>
+      <c r="E178">
+        <v>24163742.910044689</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>497</v>
+      </c>
+      <c r="B179" t="s">
+        <v>90</v>
+      </c>
+      <c r="C179" t="s">
+        <v>94</v>
+      </c>
+      <c r="E179">
+        <v>14907237.44476191</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>497</v>
+      </c>
+      <c r="B180" t="s">
+        <v>90</v>
+      </c>
+      <c r="C180" t="s">
+        <v>95</v>
+      </c>
+      <c r="E180">
+        <v>18899174.40615667</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>497</v>
+      </c>
+      <c r="B181" t="s">
+        <v>90</v>
+      </c>
+      <c r="C181" t="s">
+        <v>96</v>
+      </c>
+      <c r="E181">
+        <v>3839645.5035856571</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>497</v>
+      </c>
+      <c r="B182" t="s">
+        <v>90</v>
+      </c>
+      <c r="C182" t="s">
+        <v>93</v>
+      </c>
+      <c r="E182">
+        <v>2740233.6539654071</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>498</v>
+      </c>
+      <c r="B183" t="s">
+        <v>90</v>
+      </c>
+      <c r="C183" t="s">
+        <v>98</v>
+      </c>
+      <c r="E183">
+        <v>22648513.31474198</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>498</v>
+      </c>
+      <c r="B184" t="s">
+        <v>90</v>
+      </c>
+      <c r="C184" t="s">
+        <v>91</v>
+      </c>
+      <c r="E184">
+        <v>23504509.507710181</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>498</v>
+      </c>
+      <c r="B185" t="s">
+        <v>90</v>
+      </c>
+      <c r="C185" t="s">
+        <v>94</v>
+      </c>
+      <c r="E185">
+        <v>12840482.784761909</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>498</v>
+      </c>
+      <c r="B186" t="s">
+        <v>90</v>
+      </c>
+      <c r="C186" t="s">
+        <v>95</v>
+      </c>
+      <c r="E186">
+        <v>20078615.347537041</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>498</v>
+      </c>
+      <c r="B187" t="s">
+        <v>90</v>
+      </c>
+      <c r="C187" t="s">
+        <v>96</v>
+      </c>
+      <c r="E187">
+        <v>3216356.398978495</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>498</v>
+      </c>
+      <c r="B188" t="s">
+        <v>90</v>
+      </c>
+      <c r="C188" t="s">
+        <v>93</v>
+      </c>
+      <c r="E188">
+        <v>2060918.427395666</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>499</v>
+      </c>
+      <c r="B189" t="s">
+        <v>90</v>
+      </c>
+      <c r="C189" t="s">
+        <v>98</v>
+      </c>
+      <c r="E189">
+        <v>22674603.910064019</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>499</v>
+      </c>
+      <c r="B190" t="s">
+        <v>90</v>
+      </c>
+      <c r="C190" t="s">
+        <v>91</v>
+      </c>
+      <c r="E190">
+        <v>23892351.16330291</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>499</v>
+      </c>
+      <c r="B191" t="s">
+        <v>90</v>
+      </c>
+      <c r="C191" t="s">
+        <v>94</v>
+      </c>
+      <c r="E191">
+        <v>12530391.504761901</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>499</v>
+      </c>
+      <c r="B192" t="s">
+        <v>90</v>
+      </c>
+      <c r="C192" t="s">
+        <v>95</v>
+      </c>
+      <c r="E192">
+        <v>17771069.282792389</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>499</v>
+      </c>
+      <c r="B193" t="s">
+        <v>90</v>
+      </c>
+      <c r="C193" t="s">
+        <v>96</v>
+      </c>
+      <c r="E193">
+        <v>3247746.489788108</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>499</v>
+      </c>
+      <c r="B194" t="s">
+        <v>90</v>
+      </c>
+      <c r="C194" t="s">
+        <v>93</v>
+      </c>
+      <c r="E194">
+        <v>3116406.8132882458</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>500</v>
+      </c>
+      <c r="B195" t="s">
+        <v>90</v>
+      </c>
+      <c r="C195" t="s">
+        <v>98</v>
+      </c>
+      <c r="E195">
+        <v>23470015.951714128</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>500</v>
+      </c>
+      <c r="B196" t="s">
+        <v>90</v>
+      </c>
+      <c r="C196" t="s">
+        <v>91</v>
+      </c>
+      <c r="E196">
+        <v>24792477.474041179</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>500</v>
+      </c>
+      <c r="B197" t="s">
+        <v>90</v>
+      </c>
+      <c r="C197" t="s">
+        <v>94</v>
+      </c>
+      <c r="E197">
+        <v>14611795.18476191</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>500</v>
+      </c>
+      <c r="B198" t="s">
+        <v>90</v>
+      </c>
+      <c r="C198" t="s">
+        <v>95</v>
+      </c>
+      <c r="E198">
+        <v>18760745.560399849</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>500</v>
+      </c>
+      <c r="B199" t="s">
+        <v>90</v>
+      </c>
+      <c r="C199" t="s">
+        <v>96</v>
+      </c>
+      <c r="E199">
+        <v>3409858.838336057</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>500</v>
+      </c>
+      <c r="B200" t="s">
+        <v>90</v>
+      </c>
+      <c r="C200" t="s">
+        <v>93</v>
+      </c>
+      <c r="E200">
+        <v>4505334.575696514</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>501</v>
+      </c>
+      <c r="B201" t="s">
+        <v>90</v>
+      </c>
+      <c r="C201" t="s">
+        <v>98</v>
+      </c>
+      <c r="E201">
+        <v>22621936.559258658</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>501</v>
+      </c>
+      <c r="B202" t="s">
+        <v>90</v>
+      </c>
+      <c r="C202" t="s">
+        <v>91</v>
+      </c>
+      <c r="E202">
+        <v>23642786.400619481</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>501</v>
+      </c>
+      <c r="B203" t="s">
+        <v>90</v>
+      </c>
+      <c r="C203" t="s">
+        <v>94</v>
+      </c>
+      <c r="E203">
+        <v>12016926.99428571</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>501</v>
+      </c>
+      <c r="B204" t="s">
+        <v>90</v>
+      </c>
+      <c r="C204" t="s">
+        <v>95</v>
+      </c>
+      <c r="E204">
+        <v>17390186.846839622</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>501</v>
+      </c>
+      <c r="B205" t="s">
+        <v>90</v>
+      </c>
+      <c r="C205" t="s">
+        <v>96</v>
+      </c>
+      <c r="E205">
+        <v>3456084.406932943</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>501</v>
+      </c>
+      <c r="B206" t="s">
+        <v>90</v>
+      </c>
+      <c r="C206" t="s">
+        <v>93</v>
+      </c>
+      <c r="E206">
+        <v>3683298.36296571</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>502</v>
+      </c>
+      <c r="B207" t="s">
+        <v>90</v>
+      </c>
+      <c r="C207" t="s">
+        <v>98</v>
+      </c>
+      <c r="E207">
+        <v>22769135.052535169</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>502</v>
+      </c>
+      <c r="B208" t="s">
+        <v>90</v>
+      </c>
+      <c r="C208" t="s">
+        <v>91</v>
+      </c>
+      <c r="E208">
+        <v>24158478.228052251</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>502</v>
+      </c>
+      <c r="B209" t="s">
+        <v>90</v>
+      </c>
+      <c r="C209" t="s">
+        <v>94</v>
+      </c>
+      <c r="E209">
+        <v>12033698.99428571</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>502</v>
+      </c>
+      <c r="B210" t="s">
+        <v>90</v>
+      </c>
+      <c r="C210" t="s">
+        <v>95</v>
+      </c>
+      <c r="E210">
+        <v>17379633.519875061</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>502</v>
+      </c>
+      <c r="B211" t="s">
+        <v>90</v>
+      </c>
+      <c r="C211" t="s">
+        <v>96</v>
+      </c>
+      <c r="E211">
+        <v>3477804.4015584351</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>502</v>
+      </c>
+      <c r="B212" t="s">
+        <v>90</v>
+      </c>
+      <c r="C212" t="s">
+        <v>93</v>
+      </c>
+      <c r="E212">
+        <v>3293437.9612455191</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>503</v>
+      </c>
+      <c r="B213" t="s">
+        <v>90</v>
+      </c>
+      <c r="C213" t="s">
+        <v>98</v>
+      </c>
+      <c r="E213">
+        <v>74718831.424577147</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>503</v>
+      </c>
+      <c r="B214" t="s">
+        <v>90</v>
+      </c>
+      <c r="C214" t="s">
+        <v>91</v>
+      </c>
+      <c r="E214">
+        <v>27331633.67587252</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>503</v>
+      </c>
+      <c r="B215" t="s">
+        <v>90</v>
+      </c>
+      <c r="C215" t="s">
+        <v>94</v>
+      </c>
+      <c r="E215">
+        <v>11529703.99428571</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>503</v>
+      </c>
+      <c r="B216" t="s">
+        <v>90</v>
+      </c>
+      <c r="C216" t="s">
+        <v>95</v>
+      </c>
+      <c r="E216">
+        <v>106066711.6235541</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>503</v>
+      </c>
+      <c r="B217" t="s">
+        <v>90</v>
+      </c>
+      <c r="C217" t="s">
+        <v>96</v>
+      </c>
+      <c r="E217">
+        <v>3598284.0393927582</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>503</v>
+      </c>
+      <c r="B218" t="s">
+        <v>90</v>
+      </c>
+      <c r="C218" t="s">
+        <v>93</v>
+      </c>
+      <c r="E218">
+        <v>1977959.772256132</v>
       </c>
     </row>
   </sheetData>
@@ -14241,34 +15602,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="51" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
     </row>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -16259,7 +17620,7 @@
         <v>293.08</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>121</v>
       </c>
@@ -16275,10 +17636,15 @@
       <c r="F148">
         <v>367746</v>
       </c>
+      <c r="G148" s="42">
+        <v>372768</v>
+      </c>
       <c r="J148" s="14">
         <v>0.95499999999999996</v>
       </c>
-      <c r="L148" s="16"/>
+      <c r="L148" s="16">
+        <v>83</v>
+      </c>
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
@@ -16344,40 +17710,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
     </row>
     <row r="3" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -23776,26 +25142,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>155</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
     </row>
     <row r="3" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -23867,30 +25233,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
     </row>
     <row r="3" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -23964,7 +25330,7 @@
   <sheetPr>
     <tabColor rgb="FF1F5464"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -23976,28 +25342,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="45" t="s">
         <v>172</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -24026,25 +25392,12 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
-        <v>46113</v>
-      </c>
-      <c r="B4" s="4">
-        <v>220000000</v>
-      </c>
-      <c r="C4" s="4">
-        <v>3229000000</v>
-      </c>
-      <c r="D4" s="4">
-        <v>129000000</v>
-      </c>
-      <c r="E4" s="4">
-        <v>9000000</v>
-      </c>
-      <c r="F4" s="4">
-        <f>220000000</f>
-        <v>220000000</v>
-      </c>
+      <c r="A4" s="11"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
         <v>181</v>
       </c>
@@ -24053,58 +25406,227 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <v>46143</v>
+      <c r="A5" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5">
+        <v>275958000</v>
+      </c>
+      <c r="C5">
+        <v>2929944000</v>
+      </c>
+      <c r="D5">
+        <v>55912000</v>
+      </c>
+      <c r="E5">
+        <v>10792000</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>46174</v>
+      <c r="A6" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6">
+        <v>281191113.35912281</v>
+      </c>
+      <c r="C6">
+        <v>2932370000</v>
+      </c>
+      <c r="D6">
+        <v>6279113.3591227718</v>
+      </c>
+      <c r="E6">
+        <v>23912000</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>46204</v>
+      <c r="A7" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7">
+        <v>293369270.19912279</v>
+      </c>
+      <c r="C7">
+        <v>2914703000</v>
+      </c>
+      <c r="D7">
+        <v>20954156.840000071</v>
+      </c>
+      <c r="E7">
+        <v>14219000</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
-        <v>46235</v>
+      <c r="A8" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8">
+        <v>293224437.35912281</v>
+      </c>
+      <c r="C8">
+        <v>2918881000</v>
+      </c>
+      <c r="D8">
+        <v>4496167.1599999517</v>
+      </c>
+      <c r="E8">
+        <v>24791000</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
-        <v>46266</v>
+      <c r="A9" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9">
+        <v>342252437.35912281</v>
+      </c>
+      <c r="C9">
+        <v>2864082000</v>
+      </c>
+      <c r="D9">
+        <v>50001000</v>
+      </c>
+      <c r="E9">
+        <v>8949000</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
-        <v>46296</v>
+      <c r="A10" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10">
+        <v>290672437.35912281</v>
+      </c>
+      <c r="C10">
+        <v>2927303000</v>
+      </c>
+      <c r="D10">
+        <v>-40718000</v>
+      </c>
+      <c r="E10">
+        <v>18089000</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
-        <v>46327</v>
+      <c r="A11" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11">
+        <v>199943437.35912281</v>
+      </c>
+      <c r="C11">
+        <v>3013583000</v>
+      </c>
+      <c r="D11">
+        <v>50596000</v>
+      </c>
+      <c r="E11">
+        <v>31759000</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
-        <v>46357</v>
+      <c r="A12" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12">
+        <v>202201437.35912281</v>
+      </c>
+      <c r="C12">
+        <v>3012051000</v>
+      </c>
+      <c r="D12">
+        <v>4947000</v>
+      </c>
+      <c r="E12">
+        <v>44506000</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
-        <v>46388</v>
+      <c r="A13" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13">
+        <v>211616807.35912281</v>
+      </c>
+      <c r="C13">
+        <v>3015317000</v>
+      </c>
+      <c r="D13">
+        <v>25242369.999999989</v>
+      </c>
+      <c r="E13">
+        <v>22803000</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
-        <v>46419</v>
+      <c r="A14" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14">
+        <v>255324437.35912281</v>
+      </c>
+      <c r="C14">
+        <v>2956578000</v>
+      </c>
+      <c r="D14">
+        <v>48141630</v>
+      </c>
+      <c r="E14">
+        <v>35050000</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
-        <v>46447</v>
+      <c r="A15" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15">
+        <v>318141437.35912281</v>
+      </c>
+      <c r="C15">
+        <v>2897764000</v>
+      </c>
+      <c r="D15">
+        <v>69367000</v>
+      </c>
+      <c r="E15">
+        <v>13194000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16">
+        <v>350113437.35912281</v>
+      </c>
+      <c r="C16">
+        <v>2872156000</v>
+      </c>
+      <c r="D16">
+        <v>42912000</v>
+      </c>
+      <c r="E16">
+        <v>49962000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17">
+        <v>220070000</v>
+      </c>
+      <c r="C17">
+        <v>3228914000</v>
+      </c>
+      <c r="D17">
+        <v>-128887000</v>
+      </c>
+      <c r="E17">
+        <v>9200000</v>
+      </c>
+      <c r="F17">
+        <v>440000000</v>
       </c>
     </row>
   </sheetData>
@@ -24121,7 +25643,7 @@
   <sheetPr>
     <tabColor rgb="FF1F5464"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -24132,26 +25654,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="45" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
         <v>184</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
     </row>
     <row r="3" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -24217,19 +25739,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
-        <v>45778</v>
+        <v>45748</v>
       </c>
       <c r="B7" t="s">
-        <v>262</v>
-      </c>
-      <c r="C7">
-        <v>2066596.35</v>
-      </c>
-      <c r="D7">
-        <v>16312677.550000001</v>
-      </c>
-      <c r="F7">
-        <v>17850118.460000001</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -24237,16 +25750,20 @@
         <v>45778</v>
       </c>
       <c r="B8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C8">
-        <v>30158962.899999999</v>
+        <v>2066596.35</v>
       </c>
       <c r="D8">
-        <v>28857133.75</v>
+        <v>16312677.550000001</v>
       </c>
       <c r="F8">
-        <v>24661530.890000001</v>
+        <v>17850118.460000001</v>
+      </c>
+      <c r="G8" s="41">
+        <f t="shared" ref="G8:G42" si="0">D8/F8</f>
+        <v>0.9138694281808144</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -24254,33 +25771,41 @@
         <v>45778</v>
       </c>
       <c r="B9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C9">
-        <v>79256317.560000002</v>
+        <v>30158962.899999999</v>
       </c>
       <c r="D9">
-        <v>82045899.170000002</v>
+        <v>28857133.75</v>
       </c>
       <c r="F9">
-        <v>79348580.739999995</v>
+        <v>24661530.890000001</v>
+      </c>
+      <c r="G9" s="41">
+        <f t="shared" si="0"/>
+        <v>1.170127429587158</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
-        <v>45809</v>
+        <v>45778</v>
       </c>
       <c r="B10" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C10">
-        <v>14045495.880000001</v>
+        <v>79256317.560000002</v>
       </c>
       <c r="D10">
-        <v>9931686.6300000008</v>
+        <v>82045899.170000002</v>
       </c>
       <c r="F10">
-        <v>2066596.35</v>
+        <v>79348580.739999995</v>
+      </c>
+      <c r="G10" s="41">
+        <f t="shared" si="0"/>
+        <v>1.0339932788317696</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -24288,16 +25813,20 @@
         <v>45809</v>
       </c>
       <c r="B11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C11">
-        <v>30689648.66</v>
+        <v>14045495.880000001</v>
       </c>
       <c r="D11">
-        <v>25309638.420000002</v>
+        <v>9931686.6300000008</v>
       </c>
       <c r="F11">
-        <v>30158962.899999999</v>
+        <v>2066596.35</v>
+      </c>
+      <c r="G11" s="41">
+        <f t="shared" si="0"/>
+        <v>4.8058183350609323</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -24305,33 +25834,41 @@
         <v>45809</v>
       </c>
       <c r="B12" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C12">
-        <v>83901856.620000005</v>
+        <v>30689648.66</v>
       </c>
       <c r="D12">
-        <v>77048147</v>
+        <v>25309638.420000002</v>
       </c>
       <c r="F12">
-        <v>79256317.560000002</v>
+        <v>30158962.899999999</v>
+      </c>
+      <c r="G12" s="41">
+        <f t="shared" si="0"/>
+        <v>0.83920785021423938</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
-        <v>45839</v>
+        <v>45809</v>
       </c>
       <c r="B13" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C13">
-        <v>17057169.390000001</v>
+        <v>83901856.620000005</v>
       </c>
       <c r="D13">
-        <v>10036217.83</v>
+        <v>77048147</v>
       </c>
       <c r="F13">
-        <v>14045495.880000001</v>
+        <v>79256317.560000002</v>
+      </c>
+      <c r="G13" s="41">
+        <f t="shared" si="0"/>
+        <v>0.97213887008656019</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -24339,16 +25876,20 @@
         <v>45839</v>
       </c>
       <c r="B14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C14">
-        <v>30545224.829999998</v>
+        <v>17057169.390000001</v>
       </c>
       <c r="D14">
-        <v>27491812.890000001</v>
+        <v>10036217.83</v>
       </c>
       <c r="F14">
-        <v>30689648.66</v>
+        <v>14045495.880000001</v>
+      </c>
+      <c r="G14" s="41">
+        <f t="shared" si="0"/>
+        <v>0.714550622900471</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -24356,475 +25897,625 @@
         <v>45839</v>
       </c>
       <c r="B15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C15">
-        <v>88962739.189999998</v>
+        <v>30545224.829999998</v>
       </c>
       <c r="D15">
-        <v>77466403.189999998</v>
+        <v>27491812.890000001</v>
       </c>
       <c r="F15">
-        <v>83901856.620000005</v>
+        <v>30689648.66</v>
+      </c>
+      <c r="G15" s="41">
+        <f t="shared" si="0"/>
+        <v>0.89580083482128725</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="B16" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C16">
-        <v>20267616.489999998</v>
+        <v>88962739.189999998</v>
       </c>
       <c r="D16">
-        <v>15144317.02</v>
+        <v>77466403.189999998</v>
       </c>
       <c r="F16">
-        <v>17057169.390000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>83901856.620000005</v>
+      </c>
+      <c r="G16" s="41">
+        <f t="shared" si="0"/>
+        <v>0.92329784239284685</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <v>45870</v>
       </c>
       <c r="B17" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C17">
-        <v>28412199.100000001</v>
+        <v>20267616.489999998</v>
       </c>
       <c r="D17">
-        <v>25741058.850000001</v>
+        <v>15144317.02</v>
       </c>
       <c r="F17">
-        <v>30545224.829999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>17057169.390000001</v>
+      </c>
+      <c r="G17" s="41">
+        <f t="shared" si="0"/>
+        <v>0.88785640065687355</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
         <v>45870</v>
       </c>
       <c r="B18" t="s">
+        <v>263</v>
+      </c>
+      <c r="C18">
+        <v>28412199.100000001</v>
+      </c>
+      <c r="D18">
+        <v>25741058.850000001</v>
+      </c>
+      <c r="F18">
+        <v>30545224.829999998</v>
+      </c>
+      <c r="G18" s="41">
+        <f t="shared" si="0"/>
+        <v>0.84271957378812334</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="12">
+        <v>45870</v>
+      </c>
+      <c r="B19" t="s">
         <v>264</v>
       </c>
-      <c r="C18">
+      <c r="C19">
         <v>82185975.519999996</v>
       </c>
-      <c r="D18">
+      <c r="D19">
         <v>79568870.730000004</v>
       </c>
-      <c r="F18">
+      <c r="F19">
         <v>88962739.189999998</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
-        <v>45901</v>
-      </c>
-      <c r="B19" t="s">
-        <v>262</v>
-      </c>
-      <c r="C19">
-        <v>18790020.489999998</v>
-      </c>
-      <c r="D19">
-        <v>89152993.390000001</v>
-      </c>
-      <c r="F19">
-        <v>20267616.489999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="41">
+        <f t="shared" si="0"/>
+        <v>0.89440670840926706</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="12">
         <v>45901</v>
       </c>
       <c r="B20" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C20">
-        <v>32320493.050000001</v>
+        <v>18790020.489999998</v>
       </c>
       <c r="D20">
-        <v>28466369.489999998</v>
+        <v>89152993.390000001</v>
       </c>
       <c r="F20">
-        <v>28412199.100000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>20267616.489999998</v>
+      </c>
+      <c r="G20" s="41">
+        <f t="shared" si="0"/>
+        <v>4.3987902294277132</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
         <v>45901</v>
       </c>
       <c r="B21" t="s">
+        <v>263</v>
+      </c>
+      <c r="C21">
+        <v>32320493.050000001</v>
+      </c>
+      <c r="D21">
+        <v>28466369.489999998</v>
+      </c>
+      <c r="F21">
+        <v>28412199.100000001</v>
+      </c>
+      <c r="G21" s="41">
+        <f t="shared" si="0"/>
+        <v>1.0019065891312862</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="12">
+        <v>45901</v>
+      </c>
+      <c r="B22" t="s">
         <v>264</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>84846832.390000001</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>76843498.579999998</v>
       </c>
-      <c r="F21">
+      <c r="F22">
         <v>82185975.519999996</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
-        <v>45931</v>
-      </c>
-      <c r="B22" t="s">
-        <v>262</v>
-      </c>
-      <c r="C22">
-        <v>88569528.640000001</v>
-      </c>
-      <c r="D22">
-        <v>36808494.689999998</v>
-      </c>
-      <c r="F22">
-        <v>18790020.489999998</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="41">
+        <f t="shared" si="0"/>
+        <v>0.93499527253649373</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
         <v>45931</v>
       </c>
       <c r="B23" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C23">
-        <v>30979551.32</v>
+        <v>88569528.640000001</v>
       </c>
       <c r="D23">
-        <v>28166980.57</v>
+        <v>36808494.689999998</v>
       </c>
       <c r="F23">
-        <v>32320493.050000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>18790020.489999998</v>
+      </c>
+      <c r="G23" s="41">
+        <f t="shared" si="0"/>
+        <v>1.9589385072565186</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
         <v>45931</v>
       </c>
       <c r="B24" t="s">
+        <v>263</v>
+      </c>
+      <c r="C24">
+        <v>30979551.32</v>
+      </c>
+      <c r="D24">
+        <v>28166980.57</v>
+      </c>
+      <c r="F24">
+        <v>32320493.050000001</v>
+      </c>
+      <c r="G24" s="41">
+        <f t="shared" si="0"/>
+        <v>0.87148981689188676</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="12">
+        <v>45931</v>
+      </c>
+      <c r="B25" t="s">
         <v>264</v>
       </c>
-      <c r="C24">
+      <c r="C25">
         <v>84900219.689999998</v>
       </c>
-      <c r="D24">
+      <c r="D25">
         <v>81265425.219999999</v>
       </c>
-      <c r="F24">
+      <c r="F25">
         <v>84846832.390000001</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
-        <v>45962</v>
-      </c>
-      <c r="B25" t="s">
-        <v>262</v>
-      </c>
-      <c r="C25">
-        <v>19647436.620000001</v>
-      </c>
-      <c r="D25">
-        <v>20864043.09</v>
-      </c>
-      <c r="F25">
-        <v>88569528.640000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="41">
+        <f t="shared" si="0"/>
+        <v>0.95778973629165087</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
         <v>45962</v>
       </c>
       <c r="B26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C26">
-        <v>30525553.379999999</v>
+        <v>19647436.620000001</v>
       </c>
       <c r="D26">
-        <v>23246969.399999999</v>
+        <v>20864043.09</v>
       </c>
       <c r="F26">
-        <v>30979551.32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>88569528.640000001</v>
+      </c>
+      <c r="G26" s="41">
+        <f t="shared" si="0"/>
+        <v>0.2355668299286548</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
         <v>45962</v>
       </c>
       <c r="B27" t="s">
+        <v>263</v>
+      </c>
+      <c r="C27">
+        <v>30525553.379999999</v>
+      </c>
+      <c r="D27">
+        <v>23246969.399999999</v>
+      </c>
+      <c r="F27">
+        <v>30979551.32</v>
+      </c>
+      <c r="G27" s="41">
+        <f t="shared" si="0"/>
+        <v>0.75039722686338761</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="12">
+        <v>45962</v>
+      </c>
+      <c r="B28" t="s">
         <v>264</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>86181657.439999998</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <v>73383143.909999996</v>
       </c>
-      <c r="F27">
+      <c r="F28">
         <v>84900219.689999998</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
-        <v>45992</v>
-      </c>
-      <c r="B28" t="s">
-        <v>262</v>
-      </c>
-      <c r="C28">
-        <v>32549525.390000001</v>
-      </c>
-      <c r="D28">
-        <v>3524217.32</v>
-      </c>
-      <c r="F28">
-        <v>19647436.620000001</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="41">
+        <f t="shared" si="0"/>
+        <v>0.86434574819649679</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="12">
         <v>45992</v>
       </c>
       <c r="B29" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C29">
-        <v>27489474.789999999</v>
+        <v>32549525.390000001</v>
       </c>
       <c r="D29">
-        <v>28384758.699999999</v>
+        <v>3524217.32</v>
       </c>
       <c r="F29">
-        <v>30525553.379999999</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19647436.620000001</v>
+      </c>
+      <c r="G29" s="41">
+        <f t="shared" si="0"/>
+        <v>0.17937288146854447</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
         <v>45992</v>
       </c>
       <c r="B30" t="s">
+        <v>263</v>
+      </c>
+      <c r="C30">
+        <v>27489474.789999999</v>
+      </c>
+      <c r="D30">
+        <v>28384758.699999999</v>
+      </c>
+      <c r="F30">
+        <v>30525553.379999999</v>
+      </c>
+      <c r="G30" s="41">
+        <f t="shared" si="0"/>
+        <v>0.92986876754206116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="12">
+        <v>45992</v>
+      </c>
+      <c r="B31" t="s">
         <v>264</v>
       </c>
-      <c r="C30">
+      <c r="C31">
         <v>97016269.129999995</v>
       </c>
-      <c r="D30">
+      <c r="D31">
         <v>79154788.859999999</v>
       </c>
-      <c r="F30">
+      <c r="F31">
         <v>86181657.439999998</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="12">
-        <v>46023</v>
-      </c>
-      <c r="B31" t="s">
-        <v>262</v>
-      </c>
-      <c r="C31">
-        <v>26532644.07</v>
-      </c>
-      <c r="D31">
-        <v>21176054.359999999</v>
-      </c>
-      <c r="F31">
-        <v>32549525.390000001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="41">
+        <f t="shared" si="0"/>
+        <v>0.91846445300855195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="12">
         <v>46023</v>
       </c>
       <c r="B32" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C32">
-        <v>28529590.02</v>
+        <v>26532644.07</v>
       </c>
       <c r="D32">
-        <v>29245043.210000001</v>
+        <v>21176054.359999999</v>
       </c>
       <c r="F32">
-        <v>27489474.789999999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+        <v>32549525.390000001</v>
+      </c>
+      <c r="G32" s="41">
+        <f t="shared" si="0"/>
+        <v>0.65057951248978252</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="12">
         <v>46023</v>
       </c>
       <c r="B33" t="s">
+        <v>263</v>
+      </c>
+      <c r="C33">
+        <v>28529590.02</v>
+      </c>
+      <c r="D33">
+        <v>29245043.210000001</v>
+      </c>
+      <c r="F33">
+        <v>27489474.789999999</v>
+      </c>
+      <c r="G33" s="41">
+        <f t="shared" si="0"/>
+        <v>1.0638632943485204</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="12">
+        <v>46023</v>
+      </c>
+      <c r="B34" t="s">
         <v>264</v>
       </c>
-      <c r="C33">
+      <c r="C34">
         <v>75193263.420000002</v>
       </c>
-      <c r="D33">
+      <c r="D34">
         <v>83046164.769999996</v>
       </c>
-      <c r="F33">
+      <c r="F34">
         <v>97016269.129999995</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
-        <v>46054</v>
-      </c>
-      <c r="B34" t="s">
-        <v>262</v>
-      </c>
-      <c r="C34">
-        <v>76739509.549999997</v>
-      </c>
-      <c r="D34">
-        <v>61515826.219999999</v>
-      </c>
-      <c r="F34">
-        <v>26532644.07</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="41">
+        <f t="shared" si="0"/>
+        <v>0.85600245726538593</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="12">
         <v>46054</v>
       </c>
       <c r="B35" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C35">
-        <v>20047689.100000001</v>
+        <v>76739509.549999997</v>
       </c>
       <c r="D35">
-        <v>23482888.739999998</v>
+        <v>61515826.219999999</v>
       </c>
       <c r="F35">
-        <v>28529590.02</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26532644.07</v>
+      </c>
+      <c r="G35" s="41">
+        <f t="shared" si="0"/>
+        <v>2.3184958897313543</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="12">
         <v>46054</v>
       </c>
       <c r="B36" t="s">
+        <v>263</v>
+      </c>
+      <c r="C36">
+        <v>20047689.100000001</v>
+      </c>
+      <c r="D36">
+        <v>23482888.739999998</v>
+      </c>
+      <c r="F36">
+        <v>28529590.02</v>
+      </c>
+      <c r="G36" s="41">
+        <f t="shared" si="0"/>
+        <v>0.82310642121172684</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="12">
+        <v>46054</v>
+      </c>
+      <c r="B37" t="s">
         <v>264</v>
       </c>
-      <c r="C36">
+      <c r="C37">
         <v>81869288.099999994</v>
       </c>
-      <c r="D36">
+      <c r="D37">
         <v>73894414.739999995</v>
       </c>
-      <c r="F36">
+      <c r="F37">
         <v>75193263.420000002</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="12">
-        <v>46082</v>
-      </c>
-      <c r="B37" t="s">
-        <v>262</v>
-      </c>
-      <c r="C37">
-        <v>22774094.170000002</v>
-      </c>
-      <c r="D37">
-        <v>43473814.829999998</v>
-      </c>
-      <c r="F37">
-        <v>76739509.549999997</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="41">
+        <f t="shared" si="0"/>
+        <v>0.982726528668597</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="12">
         <v>46082</v>
       </c>
       <c r="B38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C38">
-        <v>22046285.789999999</v>
+        <v>22774094.170000002</v>
       </c>
       <c r="D38">
-        <v>27194505.539999999</v>
+        <v>43473814.829999998</v>
       </c>
       <c r="F38">
-        <v>20047689.100000001</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>76739509.549999997</v>
+      </c>
+      <c r="G38" s="41">
+        <f t="shared" si="0"/>
+        <v>0.56651150215749591</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="12">
         <v>46082</v>
       </c>
       <c r="B39" t="s">
+        <v>263</v>
+      </c>
+      <c r="C39">
+        <v>22046285.789999999</v>
+      </c>
+      <c r="D39">
+        <v>27194505.539999999</v>
+      </c>
+      <c r="F39">
+        <v>20047689.100000001</v>
+      </c>
+      <c r="G39" s="41">
+        <f t="shared" si="0"/>
+        <v>1.3564907857634323</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="12">
+        <v>46082</v>
+      </c>
+      <c r="B40" t="s">
         <v>264</v>
       </c>
-      <c r="C39">
+      <c r="C40">
         <v>85623111.299999997</v>
       </c>
-      <c r="D39">
+      <c r="D40">
         <v>76367933.879999995</v>
       </c>
-      <c r="F39">
+      <c r="F40">
         <v>81869288.099999994</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
-        <v>46113</v>
-      </c>
-      <c r="B40" t="s">
-        <v>262</v>
-      </c>
-      <c r="C40">
-        <v>53100767.329999998</v>
-      </c>
-      <c r="D40">
-        <v>23125919.989999998</v>
-      </c>
-      <c r="F40">
-        <v>22774094.170000002</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="41">
+        <f t="shared" si="0"/>
+        <v>0.93280319949429247</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="12">
         <v>46113</v>
       </c>
       <c r="B41" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C41">
-        <v>20927894.440000001</v>
+        <v>53100767.329999998</v>
       </c>
       <c r="D41">
-        <v>31679903.66</v>
+        <v>23125919.989999998</v>
       </c>
       <c r="F41">
-        <v>22046285.789999999</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22774094.170000002</v>
+      </c>
+      <c r="G41" s="41">
+        <f t="shared" si="0"/>
+        <v>1.0154485099329857</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="12">
         <v>46113</v>
       </c>
       <c r="B42" t="s">
+        <v>263</v>
+      </c>
+      <c r="C42">
+        <v>20927894.440000001</v>
+      </c>
+      <c r="D42">
+        <v>31679903.66</v>
+      </c>
+      <c r="F42">
+        <v>22046285.789999999</v>
+      </c>
+      <c r="G42" s="41">
+        <f t="shared" si="0"/>
+        <v>1.4369723753816948</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="12">
+        <v>46113</v>
+      </c>
+      <c r="B43" t="s">
         <v>264</v>
       </c>
-      <c r="C42">
+      <c r="C43">
         <v>76634788.340000004</v>
       </c>
-      <c r="D42">
+      <c r="D43">
         <v>81409360.709999993</v>
       </c>
-      <c r="F42">
+      <c r="F43">
         <v>85623111.299999997</v>
+      </c>
+      <c r="G43" s="41">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="12">
+        <v>46113</v>
+      </c>
+      <c r="B44" t="s">
+        <v>261</v>
+      </c>
+      <c r="D44">
+        <v>31408268.690000001</v>
+      </c>
+      <c r="F44">
+        <f>D44/G44</f>
+        <v>32147664.984646879</v>
+      </c>
+      <c r="G44" s="41">
+        <v>0.97699999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>